<commit_message>
Cross-check nižších národních soutěží proti PDF (CZE1+CZE2_3): 137 oprav
verify_vs_pdf.py rozšířen: pooluje top + DS PDF, kontroluje všechny národní listy
(^\d0_, krajské vyjma). Opraveno 137 buněk (V/R/P, PTS, drobné GF:GA) v 1./2. lize
a divizích (éra <2000).

Pojistky proti špatným shodám:
- pass-1: jen přesná shoda (GP,GF,GA) -> oprava V/R/P + PTS=2V+R (ne-přenosové bloky)
- pass-2: GF:GA dle jednoznačné shody V/R/P, jen je-li 1 půlka skóre přesná nebo
  oboustranný rozdíl <=4 (podezřelé velké skoky se nehádají, jen hlásí)

223 řádků k ověření (bez shody: krajské finále/moderní éra/mezery). Extraliga beze
změny (2-1-0 čistá). MASTER_REPORT aktualizován.
</commit_message>
<xml_diff>
--- a/data/S1965_66_FINAL.xlsx
+++ b/data/S1965_66_FINAL.xlsx
@@ -55529,7 +55529,7 @@
         <v>20</v>
       </c>
       <c r="J9" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -55537,7 +55537,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="M9" t="n">
         <v>15</v>

</xml_diff>

<commit_message>
Systematicky doplnit chybějící M badge u pre-1986 mistrů (z META/MASTER_REPORT)
20 sezón postrádalo M badge v tabulce (mistr byl jen v META). Doplněn M na řádek
mistra (preferenčně finálový blok): 1954/55 RH Brno, 1965/66 ZKL Brno, 1966-71
+1973/74+1981-84 Dukla Jihlava, 1974/75+1976/77+1979/80 SONP Kladno, 1978/79 Slovan
Bratislava, 1980/81 Vítkovice, 1985/86 VSŽ Košice.

Ověřeno webem u sporných: 1970/71 = Dukla Jihlava (porazil ZKL Brno ve finále;
MASTER_REPORT 'ZKL Brno' byl chybný, data správně). Všechny pre-1986 sezóny nyní
mají M badge na mistrovi.
</commit_message>
<xml_diff>
--- a/data/S1965_66_FINAL.xlsx
+++ b/data/S1965_66_FINAL.xlsx
@@ -714,6 +714,11 @@
           <t>ZKL Brno</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
       <c r="F4" t="n">
         <v>36</v>
       </c>
@@ -19536,8 +19541,6 @@
           <t>NODE_S1965_66_0001</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -19593,8 +19596,6 @@
           <t>NODE_S1965_66_0001</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -20246,7 +20247,6 @@
           <t>NODE_S1965_66_0023</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -20297,8 +20297,6 @@
           <t>NODE_S1965_66_0019</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -20537,8 +20535,6 @@
           <t>NODE_S1965_66_0024</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -21118,8 +21114,6 @@
           <t>NODE_S1965_66_0024</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr"/>
-      <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -21662,8 +21656,6 @@
           <t>NODE_S1965_66_0049</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -21892,8 +21884,6 @@
           <t>NODE_S1965_66_0050</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -22132,8 +22122,6 @@
           <t>NODE_S1965_66_0059</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
       <c r="I64" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -22790,8 +22778,6 @@
           <t>NODE_S1965_66_0073</t>
         </is>
       </c>
-      <c r="G78" t="inlineStr"/>
-      <c r="H78" t="inlineStr"/>
       <c r="I78" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -23312,8 +23298,6 @@
           <t>NODE_S1965_66_0084</t>
         </is>
       </c>
-      <c r="G89" t="inlineStr"/>
-      <c r="H89" t="inlineStr"/>
       <c r="I89" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -23448,8 +23432,6 @@
           <t>NODE_S1965_66_0084</t>
         </is>
       </c>
-      <c r="G92" t="inlineStr"/>
-      <c r="H92" t="inlineStr"/>
       <c r="I92" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -23500,8 +23482,6 @@
           <t>NODE_S1965_66_0084</t>
         </is>
       </c>
-      <c r="G93" t="inlineStr"/>
-      <c r="H93" t="inlineStr"/>
       <c r="I93" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -24375,8 +24355,6 @@
           <t>NODE_S1965_66_0101</t>
         </is>
       </c>
-      <c r="G113" t="inlineStr"/>
-      <c r="H113" t="inlineStr"/>
       <c r="I113" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -24427,8 +24405,6 @@
           <t>NODE_S1965_66_0101</t>
         </is>
       </c>
-      <c r="G114" t="inlineStr"/>
-      <c r="H114" t="inlineStr"/>
       <c r="I114" t="inlineStr">
         <is>
           <t>2-1-0</t>
@@ -54846,7 +54822,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -55050,6 +55026,18 @@
       <c r="B17" t="inlineStr">
         <is>
           <t>Motorlet B nemohl postoupit, proto postoupila Dukla Písek. V severočeské větvi šlo po odmítnutí Chomutova B do kvalifikace Ústí nad Labem. Ve středoslovenské větvi šla místo Banské Bystrice B do kvalifikace Dubnica nad Váhom.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>mistr</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ZKL Brno</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rozšířit verify_vs_pdf na oblastní + KVAL: 25 oprav z DS PDF
verify_vs_pdf.py nyní diffuje i listy 20_oblastni a KVAL proti DS PDF (nejen
nejvyšší soutěž). Najdeno+opraveno 25 drobných nesrovnalostí (GF:GA překlepy,
pár V/R/P) napříč sezónami — s pojistkou (jedno číslo přesně / rozdíl ≤4).
303 řádků k ověření (neúplné rozpisy v datech vs PDF — k ruční kontrole).
Tím odhaleny i 'balancované ale odlišné' případy, které interní check minul.
</commit_message>
<xml_diff>
--- a/data/S1965_66_FINAL.xlsx
+++ b/data/S1965_66_FINAL.xlsx
@@ -58930,7 +58930,7 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="M10" t="n">
         <v>3</v>
@@ -59023,13 +59023,13 @@
         <v>4</v>
       </c>
       <c r="G12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H12" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J12" t="n">
         <v>19</v>

</xml_diff>